<commit_message>
make project modular isolate proforma
</commit_message>
<xml_diff>
--- a/catafactuapp1.xlsx
+++ b/catafactuapp1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/h.boukhalfa/Desktop/catafactuapp/proforma-app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/h.boukhalfa/Desktop/catafactuappfull/catafactu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E45A57E-9FD4-A642-8C2A-0D2E1126484F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91903EB7-641E-D645-BA73-69142B06D1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1400" yWindow="740" windowWidth="28000" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>prix-gros</t>
   </si>
   <si>
-    <t>prix-detaille</t>
-  </si>
-  <si>
     <t>UNI-COLOR</t>
   </si>
   <si>
@@ -765,6 +762,9 @@
   </si>
   <si>
     <t>TABLE RONDE PLIABLE (PARTENAIRE) 1,80 M</t>
+  </si>
+  <si>
+    <t>prix-détail</t>
   </si>
 </sst>
 </file>
@@ -1628,67 +1628,67 @@
         <v>8</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Z1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="4" t="s">
+      <c r="AA1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AC1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AD1" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="AD1" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="AE1" s="8"/>
       <c r="AF1" s="8"/>
@@ -1707,17 +1707,17 @@
     </row>
     <row r="2" spans="1:44" ht="207" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" s="10">
         <f t="shared" ref="B2:B16" si="0">SUM(K2:AC2)</f>
         <v>8</v>
       </c>
       <c r="C2" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>32</v>
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
@@ -1806,17 +1806,17 @@
     </row>
     <row r="3" spans="1:44" ht="204" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="16"/>
       <c r="F3" s="16"/>
@@ -1905,17 +1905,17 @@
     </row>
     <row r="4" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C4" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>36</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>37</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
@@ -2004,17 +2004,17 @@
     </row>
     <row r="5" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B5" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="16" t="s">
         <v>36</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>37</v>
       </c>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
@@ -2103,17 +2103,17 @@
     </row>
     <row r="6" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
@@ -2202,17 +2202,17 @@
     </row>
     <row r="7" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
@@ -2301,17 +2301,17 @@
     </row>
     <row r="8" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -2400,17 +2400,17 @@
     </row>
     <row r="9" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="15">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
@@ -2499,17 +2499,17 @@
     </row>
     <row r="10" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="15">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
@@ -2598,17 +2598,17 @@
     </row>
     <row r="11" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="C11" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="20" t="s">
         <v>49</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>50</v>
       </c>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
@@ -2697,17 +2697,17 @@
     </row>
     <row r="12" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
@@ -2796,17 +2796,17 @@
     </row>
     <row r="13" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
@@ -2895,17 +2895,17 @@
     </row>
     <row r="14" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B14" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
@@ -2994,17 +2994,17 @@
     </row>
     <row r="15" spans="1:44" ht="156.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E15" s="23"/>
       <c r="F15" s="24"/>
@@ -3093,20 +3093,20 @@
     </row>
     <row r="16" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="15">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="16" t="s">
         <v>59</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>60</v>
       </c>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
@@ -3194,14 +3194,14 @@
     </row>
     <row r="17" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
@@ -3290,20 +3290,20 @@
     </row>
     <row r="18" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="15">
         <f t="shared" ref="B18:B31" si="1">SUM(K18:AC18)</f>
         <v>20</v>
       </c>
       <c r="C18" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="16" t="s">
         <v>64</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>65</v>
       </c>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
@@ -3391,20 +3391,20 @@
     </row>
     <row r="19" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" s="15">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="C19" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="16" t="s">
         <v>67</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>68</v>
       </c>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
@@ -3492,17 +3492,17 @@
     </row>
     <row r="20" spans="1:44" ht="177.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="15">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
@@ -3574,7 +3574,7 @@
         <v>0</v>
       </c>
       <c r="AD20" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AE20" s="18"/>
       <c r="AF20" s="18"/>
@@ -3593,17 +3593,17 @@
     </row>
     <row r="21" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B21" s="15">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -3694,17 +3694,17 @@
     </row>
     <row r="22" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
@@ -3793,17 +3793,17 @@
     </row>
     <row r="23" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" s="15">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
@@ -3892,17 +3892,17 @@
     </row>
     <row r="24" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24" s="15">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
@@ -3991,17 +3991,17 @@
     </row>
     <row r="25" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B25" s="15">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="C25" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" s="16" t="s">
         <v>81</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>82</v>
       </c>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
@@ -4090,17 +4090,17 @@
     </row>
     <row r="26" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B26" s="15">
         <f t="shared" si="1"/>
         <v>101</v>
       </c>
       <c r="C26" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" s="16" t="s">
         <v>84</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>85</v>
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="28"/>
@@ -4189,17 +4189,17 @@
     </row>
     <row r="27" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B27" s="15">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D27" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
@@ -4288,17 +4288,17 @@
     </row>
     <row r="28" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B28" s="15">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
@@ -4387,20 +4387,20 @@
     </row>
     <row r="29" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B29" s="15">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
       <c r="C29" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E29" s="16" t="s">
         <v>91</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>92</v>
       </c>
       <c r="F29" s="16"/>
       <c r="G29" s="16"/>
@@ -4488,20 +4488,20 @@
     </row>
     <row r="30" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B30" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="C30" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30" s="16" t="s">
         <v>94</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E30" s="16" t="s">
-        <v>95</v>
       </c>
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
@@ -4589,20 +4589,20 @@
     </row>
     <row r="31" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B31" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
@@ -4690,17 +4690,17 @@
     </row>
     <row r="32" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B32" s="30"/>
       <c r="C32" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="D32" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="D32" s="31" t="s">
+      <c r="E32" s="31" t="s">
         <v>100</v>
-      </c>
-      <c r="E32" s="31" t="s">
-        <v>101</v>
       </c>
       <c r="F32" s="32"/>
       <c r="G32" s="16"/>
@@ -4750,17 +4750,17 @@
     </row>
     <row r="33" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="29" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="30"/>
       <c r="C33" s="31" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D33" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="E33" s="31" t="s">
         <v>100</v>
-      </c>
-      <c r="E33" s="31" t="s">
-        <v>101</v>
       </c>
       <c r="F33" s="32"/>
       <c r="G33" s="16"/>
@@ -4810,20 +4810,20 @@
     </row>
     <row r="34" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B34" s="15">
         <f>SUM(K34:AC34)</f>
         <v>10</v>
       </c>
       <c r="C34" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E34" s="16" t="s">
         <v>105</v>
-      </c>
-      <c r="D34" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E34" s="16" t="s">
-        <v>106</v>
       </c>
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
@@ -4911,17 +4911,17 @@
     </row>
     <row r="35" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B35" s="37"/>
       <c r="C35" s="38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F35" s="16"/>
       <c r="G35" s="39"/>
@@ -4971,20 +4971,20 @@
     </row>
     <row r="36" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B36" s="15">
         <f>SUM(K36:AC36)</f>
         <v>6</v>
       </c>
       <c r="C36" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36" s="20" t="s">
         <v>109</v>
-      </c>
-      <c r="D36" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E36" s="20" t="s">
-        <v>110</v>
       </c>
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
@@ -5072,14 +5072,14 @@
     </row>
     <row r="37" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B37" s="15"/>
       <c r="C37" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D37" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37" s="16"/>
       <c r="F37" s="16"/>
@@ -5130,17 +5130,17 @@
     </row>
     <row r="38" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B38" s="15">
         <f t="shared" ref="B38:B66" si="2">SUM(K38:AC38)</f>
         <v>1</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E38" s="16"/>
       <c r="F38" s="16"/>
@@ -5229,17 +5229,17 @@
     </row>
     <row r="39" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B39" s="15">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
@@ -5311,7 +5311,7 @@
         <v>0</v>
       </c>
       <c r="AD39" s="17" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AE39" s="18"/>
       <c r="AF39" s="18"/>
@@ -5330,20 +5330,20 @@
     </row>
     <row r="40" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B40" s="15">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="C40" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E40" s="16" t="s">
         <v>119</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E40" s="16" t="s">
-        <v>120</v>
       </c>
       <c r="F40" s="16"/>
       <c r="G40" s="16"/>
@@ -5431,20 +5431,20 @@
     </row>
     <row r="41" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B41" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D41" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F41" s="16"/>
       <c r="G41" s="16"/>
@@ -5532,20 +5532,20 @@
     </row>
     <row r="42" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B42" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F42" s="16"/>
       <c r="G42" s="16"/>
@@ -5633,17 +5633,17 @@
     </row>
     <row r="43" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B43" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C43" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="D43" s="16" t="s">
         <v>126</v>
-      </c>
-      <c r="D43" s="16" t="s">
-        <v>127</v>
       </c>
       <c r="E43" s="16"/>
       <c r="F43" s="16"/>
@@ -5732,17 +5732,17 @@
     </row>
     <row r="44" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B44" s="15">
         <f t="shared" si="2"/>
         <v>40750</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E44" s="16"/>
       <c r="F44" s="40"/>
@@ -5835,17 +5835,17 @@
     </row>
     <row r="45" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B45" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E45" s="16"/>
       <c r="F45" s="40"/>
@@ -5934,17 +5934,17 @@
     </row>
     <row r="46" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B46" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E46" s="16"/>
       <c r="F46" s="40"/>
@@ -6033,17 +6033,17 @@
     </row>
     <row r="47" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B47" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D47" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E47" s="16"/>
       <c r="F47" s="40"/>
@@ -6132,17 +6132,17 @@
     </row>
     <row r="48" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B48" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D48" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E48" s="16"/>
       <c r="F48" s="40"/>
@@ -6231,17 +6231,17 @@
     </row>
     <row r="49" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B49" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E49" s="16"/>
       <c r="F49" s="16"/>
@@ -6330,17 +6330,17 @@
     </row>
     <row r="50" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B50" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D50" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E50" s="16"/>
       <c r="F50" s="16"/>
@@ -6429,17 +6429,17 @@
     </row>
     <row r="51" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B51" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E51" s="16"/>
       <c r="F51" s="16"/>
@@ -6528,17 +6528,17 @@
     </row>
     <row r="52" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B52" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D52" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E52" s="16"/>
       <c r="F52" s="16"/>
@@ -6627,17 +6627,17 @@
     </row>
     <row r="53" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B53" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D53" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E53" s="16"/>
       <c r="F53" s="16"/>
@@ -6726,17 +6726,17 @@
     </row>
     <row r="54" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B54" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C54" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D54" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E54" s="16"/>
       <c r="F54" s="16"/>
@@ -6825,17 +6825,17 @@
     </row>
     <row r="55" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B55" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C55" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D55" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E55" s="16"/>
       <c r="F55" s="16"/>
@@ -6924,17 +6924,17 @@
     </row>
     <row r="56" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B56" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C56" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D56" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E56" s="16"/>
       <c r="F56" s="16"/>
@@ -7023,17 +7023,17 @@
     </row>
     <row r="57" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B57" s="15">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E57" s="16"/>
       <c r="F57" s="16"/>
@@ -7122,17 +7122,17 @@
     </row>
     <row r="58" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B58" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E58" s="16"/>
       <c r="F58" s="16"/>
@@ -7221,17 +7221,17 @@
     </row>
     <row r="59" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B59" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D59" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E59" s="16"/>
       <c r="F59" s="16"/>
@@ -7320,17 +7320,17 @@
     </row>
     <row r="60" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="14" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B60" s="15">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D60" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E60" s="16"/>
       <c r="F60" s="16"/>
@@ -7419,17 +7419,17 @@
     </row>
     <row r="61" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B61" s="15">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="C61" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D61" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E61" s="16"/>
       <c r="F61" s="16"/>
@@ -7518,17 +7518,17 @@
     </row>
     <row r="62" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B62" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C62" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D62" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E62" s="16"/>
       <c r="F62" s="16"/>
@@ -7617,17 +7617,17 @@
     </row>
     <row r="63" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A63" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B63" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C63" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D63" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E63" s="16"/>
       <c r="F63" s="16"/>
@@ -7716,17 +7716,17 @@
     </row>
     <row r="64" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A64" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B64" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C64" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D64" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E64" s="16"/>
       <c r="F64" s="16"/>
@@ -7815,17 +7815,17 @@
     </row>
     <row r="65" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B65" s="15">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C65" s="16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D65" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E65" s="16"/>
       <c r="F65" s="16"/>
@@ -7914,17 +7914,17 @@
     </row>
     <row r="66" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="14" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B66" s="15">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D66" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E66" s="16"/>
       <c r="F66" s="16"/>
@@ -8013,16 +8013,16 @@
     </row>
     <row r="67" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A67" s="14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B67" s="15">
         <v>4</v>
       </c>
       <c r="C67" s="16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E67" s="16"/>
       <c r="F67" s="16"/>
@@ -8056,7 +8056,7 @@
       <c r="AB67" s="17"/>
       <c r="AC67" s="17"/>
       <c r="AD67" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AE67" s="18"/>
       <c r="AF67" s="18"/>
@@ -8075,16 +8075,16 @@
     </row>
     <row r="68" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" s="15">
         <v>1</v>
       </c>
       <c r="C68" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D68" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E68" s="16"/>
       <c r="F68" s="16"/>
@@ -8118,7 +8118,7 @@
       <c r="AB68" s="17"/>
       <c r="AC68" s="17"/>
       <c r="AD68" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AE68" s="18"/>
       <c r="AF68" s="18"/>
@@ -8137,17 +8137,17 @@
     </row>
     <row r="69" spans="1:44" ht="156.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A69" s="45" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B69" s="15">
         <f t="shared" ref="B69:B70" si="3">SUM(K69:AC69)</f>
         <v>0</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E69" s="15"/>
       <c r="F69" s="46"/>
@@ -8198,17 +8198,17 @@
     </row>
     <row r="70" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A70" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B70" s="15">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="C70" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D70" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E70" s="16"/>
       <c r="F70" s="16"/>
@@ -8297,14 +8297,14 @@
     </row>
     <row r="71" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A71" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B71" s="15"/>
       <c r="C71" s="20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D71" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E71" s="16"/>
       <c r="F71" s="16"/>
@@ -8355,17 +8355,17 @@
     </row>
     <row r="72" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B72" s="15">
         <f t="shared" ref="B72:B85" si="4">SUM(K72:AC72)</f>
         <v>1</v>
       </c>
       <c r="C72" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D72" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E72" s="16"/>
       <c r="F72" s="16"/>
@@ -8454,17 +8454,17 @@
     </row>
     <row r="73" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B73" s="15">
         <f t="shared" si="4"/>
         <v>8</v>
       </c>
       <c r="C73" s="16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D73" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E73" s="16"/>
       <c r="F73" s="16"/>
@@ -8553,17 +8553,17 @@
     </row>
     <row r="74" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A74" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B74" s="15">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="C74" s="16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E74" s="16"/>
       <c r="F74" s="16"/>
@@ -8652,17 +8652,17 @@
     </row>
     <row r="75" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A75" s="14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B75" s="15">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="C75" s="16" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D75" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E75" s="16"/>
       <c r="F75" s="16"/>
@@ -8751,17 +8751,17 @@
     </row>
     <row r="76" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A76" s="14" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B76" s="15">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
       <c r="C76" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D76" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E76" s="16"/>
       <c r="F76" s="16"/>
@@ -8850,17 +8850,17 @@
     </row>
     <row r="77" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A77" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B77" s="15">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="C77" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D77" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E77" s="16"/>
       <c r="F77" s="16"/>
@@ -8949,17 +8949,17 @@
     </row>
     <row r="78" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A78" s="14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B78" s="15">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="C78" s="16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D78" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E78" s="16"/>
       <c r="F78" s="16"/>
@@ -9048,17 +9048,17 @@
     </row>
     <row r="79" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A79" s="14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B79" s="15">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="C79" s="16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D79" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E79" s="16"/>
       <c r="F79" s="16"/>
@@ -9147,17 +9147,17 @@
     </row>
     <row r="80" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A80" s="14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B80" s="15">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="C80" s="16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D80" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E80" s="16"/>
       <c r="F80" s="16"/>
@@ -9246,17 +9246,17 @@
     </row>
     <row r="81" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A81" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B81" s="15">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="C81" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D81" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E81" s="16"/>
       <c r="F81" s="16"/>
@@ -9345,17 +9345,17 @@
     </row>
     <row r="82" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A82" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B82" s="15">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D82" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E82" s="16"/>
       <c r="F82" s="16"/>
@@ -9427,7 +9427,7 @@
         <v>0</v>
       </c>
       <c r="AD82" s="17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AE82" s="18"/>
       <c r="AF82" s="18"/>
@@ -9446,17 +9446,17 @@
     </row>
     <row r="83" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A83" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B83" s="15">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="C83" s="16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D83" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E83" s="16"/>
       <c r="F83" s="16"/>
@@ -9478,7 +9478,7 @@
         <v>0</v>
       </c>
       <c r="N83" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O83" s="17">
         <v>0</v>
@@ -9526,7 +9526,7 @@
         <v>0</v>
       </c>
       <c r="AD83" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AE83" s="18"/>
       <c r="AF83" s="18"/>
@@ -9545,17 +9545,17 @@
     </row>
     <row r="84" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A84" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B84" s="15">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="C84" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D84" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E84" s="16"/>
       <c r="F84" s="16"/>
@@ -9644,17 +9644,17 @@
     </row>
     <row r="85" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A85" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B85" s="15">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="C85" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D85" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E85" s="16"/>
       <c r="F85" s="16"/>
@@ -9743,17 +9743,17 @@
     </row>
     <row r="86" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A86" s="14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B86" s="47"/>
       <c r="C86" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="D86" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E86" s="16" t="s">
         <v>200</v>
-      </c>
-      <c r="D86" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E86" s="16" t="s">
-        <v>201</v>
       </c>
       <c r="F86" s="16"/>
       <c r="G86" s="16"/>
@@ -9803,14 +9803,14 @@
     </row>
     <row r="87" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A87" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B87" s="51"/>
       <c r="C87" s="19" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D87" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E87" s="19"/>
       <c r="F87" s="19"/>
@@ -9861,17 +9861,17 @@
     </row>
     <row r="88" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A88" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B88" s="15">
         <f t="shared" ref="B88:B94" si="5">SUM(K88:AC88)</f>
         <v>6</v>
       </c>
       <c r="C88" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D88" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E88" s="16"/>
       <c r="F88" s="16"/>
@@ -9960,17 +9960,17 @@
     </row>
     <row r="89" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A89" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B89" s="15">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="C89" s="16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D89" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E89" s="16"/>
       <c r="F89" s="16"/>
@@ -9979,7 +9979,7 @@
         <v>3700</v>
       </c>
       <c r="I89" s="16" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J89" s="16">
         <v>4200</v>
@@ -10059,17 +10059,17 @@
     </row>
     <row r="90" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A90" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B90" s="15">
         <f t="shared" si="5"/>
         <v>9</v>
       </c>
       <c r="C90" s="16" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D90" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E90" s="16"/>
       <c r="F90" s="16"/>
@@ -10158,17 +10158,17 @@
     </row>
     <row r="91" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A91" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B91" s="15">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="C91" s="16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D91" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E91" s="16"/>
       <c r="F91" s="16"/>
@@ -10257,17 +10257,17 @@
     </row>
     <row r="92" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B92" s="15">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="C92" s="16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D92" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E92" s="16"/>
       <c r="F92" s="16"/>
@@ -10356,17 +10356,17 @@
     </row>
     <row r="93" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B93" s="15">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="C93" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D93" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E93" s="16"/>
       <c r="F93" s="16"/>
@@ -10387,7 +10387,7 @@
         <v>0</v>
       </c>
       <c r="M93" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N93" s="17">
         <v>2</v>
@@ -10455,17 +10455,17 @@
     </row>
     <row r="94" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B94" s="15">
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
       <c r="C94" s="17" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D94" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E94" s="17"/>
       <c r="F94" s="24"/>
@@ -10554,14 +10554,14 @@
     </row>
     <row r="95" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="17" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B95" s="15"/>
       <c r="C95" s="17" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D95" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E95" s="23"/>
       <c r="F95" s="17"/>
@@ -10612,16 +10612,16 @@
     </row>
     <row r="96" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="17" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B96" s="15">
         <v>36</v>
       </c>
       <c r="C96" s="23" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D96" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E96" s="23"/>
       <c r="F96" s="17"/>
@@ -10661,7 +10661,7 @@
       <c r="AB96" s="17"/>
       <c r="AC96" s="17"/>
       <c r="AD96" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AE96" s="26"/>
       <c r="AF96" s="26"/>
@@ -10680,16 +10680,16 @@
     </row>
     <row r="97" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B97" s="23">
         <v>0</v>
       </c>
       <c r="C97" s="54" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D97" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E97" s="17"/>
       <c r="F97" s="17"/>
@@ -10742,16 +10742,16 @@
     </row>
     <row r="98" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="56" t="s">
+        <v>220</v>
+      </c>
+      <c r="B98" s="23">
+        <v>0</v>
+      </c>
+      <c r="C98" s="57" t="s">
         <v>221</v>
       </c>
-      <c r="B98" s="23">
-        <v>0</v>
-      </c>
-      <c r="C98" s="57" t="s">
-        <v>222</v>
-      </c>
       <c r="D98" s="58" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E98" s="18"/>
       <c r="F98" s="59"/>
@@ -10804,16 +10804,16 @@
     </row>
     <row r="99" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="62" t="s">
+        <v>222</v>
+      </c>
+      <c r="B99" s="23">
+        <v>0</v>
+      </c>
+      <c r="C99" s="57" t="s">
         <v>223</v>
       </c>
-      <c r="B99" s="23">
-        <v>0</v>
-      </c>
-      <c r="C99" s="57" t="s">
-        <v>224</v>
-      </c>
       <c r="D99" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E99" s="18"/>
       <c r="F99" s="59"/>
@@ -10866,17 +10866,17 @@
     </row>
     <row r="100" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="62" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B100" s="23"/>
       <c r="C100" s="57" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D100" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E100" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F100" s="59"/>
       <c r="G100" s="17"/>
@@ -10926,19 +10926,19 @@
     </row>
     <row r="101" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="62" t="s">
+        <v>226</v>
+      </c>
+      <c r="B101" s="23">
+        <v>0</v>
+      </c>
+      <c r="C101" s="57" t="s">
         <v>227</v>
       </c>
-      <c r="B101" s="23">
-        <v>0</v>
-      </c>
-      <c r="C101" s="57" t="s">
-        <v>228</v>
-      </c>
       <c r="D101" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E101" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F101" s="59"/>
       <c r="G101" s="17"/>
@@ -10988,17 +10988,17 @@
     </row>
     <row r="102" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B102" s="66"/>
       <c r="C102" s="57" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D102" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E102" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F102" s="59"/>
       <c r="G102" s="67"/>
@@ -11048,17 +11048,17 @@
     </row>
     <row r="103" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B103" s="66"/>
       <c r="C103" s="57" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D103" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E103" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F103" s="59"/>
       <c r="G103" s="67"/>
@@ -11104,17 +11104,17 @@
     </row>
     <row r="104" spans="1:44" ht="159" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B104" s="66"/>
       <c r="C104" s="57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D104" s="63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E104" s="65" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F104" s="59"/>
       <c r="G104" s="67"/>
@@ -13617,7 +13617,7 @@
       <formula>LEN(TRIM(G1))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18:J100 H1:J16">
+  <conditionalFormatting sqref="H1:J16 H18:J100">
     <cfRule type="notContainsBlanks" dxfId="0" priority="3">
       <formula>LEN(TRIM(H1))&gt;0</formula>
     </cfRule>

</xml_diff>

<commit_message>
image working in both pdf and form but needs improvement
</commit_message>
<xml_diff>
--- a/catafactuapp1.xlsx
+++ b/catafactuapp1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/h.boukhalfa/Desktop/catafactuappfull/catafactu/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB51DE7-E598-D74B-9E63-80CD384B4C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8BC8B7-89FA-774F-8397-80F8684DBC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3580" yWindow="1640" windowWidth="28280" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="740" windowWidth="28280" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1827,7 +1827,7 @@
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="25.1640625" customWidth="1"/>
     <col min="7" max="7" width="102" customWidth="1"/>
-    <col min="8" max="8" width="65" customWidth="1"/>
+    <col min="8" max="8" width="111.33203125" customWidth="1"/>
     <col min="9" max="32" width="23.33203125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>